<commit_message>
Validate Android build, verify offline transport and finalize the 103-item roadmap
</commit_message>
<xml_diff>
--- a/docs/FranchiseGuide_Reste_a_faire.xlsx
+++ b/docs/FranchiseGuide_Reste_a_faire.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="R14d577a20f6f4ac1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Travaux" sheetId="2" r:id="Re77b990573df48fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" r:id="R17cda62ef9f74bee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Travaux" sheetId="2" r:id="R22666a5a9e304976"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -592,7 +592,7 @@
       </x:c>
       <x:c r="C7" s="21" t="n">
         <x:f>C6-C8</x:f>
-        <x:v>95</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="D7" s="2"/>
       <x:c r="E7" s="2"/>
@@ -602,7 +602,7 @@
       </x:c>
       <x:c r="H7" s="17" t="n">
         <x:f>COUNTIFS('Travaux'!$B$8:$B$1000,"P0",'Travaux'!$C$8:$C$1000,"&lt;&gt;Terminé")</x:f>
-        <x:v>23</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="I7" s="2"/>
       <x:c r="J7" s="2"/>
@@ -614,7 +614,7 @@
       </x:c>
       <x:c r="C8" s="17" t="n">
         <x:f>COUNTIFS('Travaux'!$C$8:$C$1000,"Terminé")</x:f>
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D8" s="2"/>
       <x:c r="E8" s="2"/>
@@ -624,7 +624,7 @@
       </x:c>
       <x:c r="H8" s="17" t="n">
         <x:f>COUNTIFS('Travaux'!$B$8:$B$1000,"P1",'Travaux'!$C$8:$C$1000,"&lt;&gt;Terminé")</x:f>
-        <x:v>59</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="I8" s="2"/>
       <x:c r="J8" s="2"/>
@@ -632,11 +632,11 @@
     <x:row r="9" ht="23" customHeight="1">
       <x:c r="A9" s="2"/>
       <x:c r="B9" s="2" t="str">
-        <x:v>Recettes à compléter</x:v>
+        <x:v>Statut « À valider »</x:v>
       </x:c>
       <x:c r="C9" s="17" t="n">
         <x:f>COUNTIFS('Travaux'!$C$8:$C$1000,"À valider")</x:f>
-        <x:v>55</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="D9" s="2"/>
       <x:c r="E9" s="2"/>
@@ -706,11 +706,11 @@
       </x:c>
       <x:c r="C13" s="17" t="n">
         <x:f>COUNTIFS('Travaux'!$D$8:$D$1000,B13,'Travaux'!$C$8:$C$1000,"&lt;&gt;Terminé")</x:f>
-        <x:v>9</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D13" s="17" t="n">
         <x:f>COUNTIFS('Travaux'!$D$8:$D$1000,B13,'Travaux'!$C$8:$C$1000,"Terminé")</x:f>
-        <x:v>0</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="E13" s="17" t="n">
         <x:f>SUM(C13:D13)</x:f>
@@ -750,7 +750,7 @@
       </x:c>
       <x:c r="H14" s="17" t="n">
         <x:f>COUNTIFS('Travaux'!$C$8:$C$1000,G14)</x:f>
-        <x:v>21</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="I14" s="2"/>
       <x:c r="J14" s="2"/>
@@ -778,7 +778,7 @@
       </x:c>
       <x:c r="H15" s="17" t="n">
         <x:f>COUNTIFS('Travaux'!$C$8:$C$1000,G15)</x:f>
-        <x:v>55</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="I15" s="2"/>
       <x:c r="J15" s="2"/>
@@ -806,7 +806,7 @@
       </x:c>
       <x:c r="H16" s="17" t="n">
         <x:f>COUNTIFS('Travaux'!$C$8:$C$1000,G16)</x:f>
-        <x:v>8</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="I16" s="2"/>
       <x:c r="J16" s="2"/>
@@ -1071,7 +1071,7 @@
     <x:row r="29" ht="23" customHeight="1">
       <x:c r="A29" s="2"/>
       <x:c r="B29" s="2" t="str">
-        <x:v>1. Vérifier Android, les comptes réels et les parcours sur les plateformes cibles.</x:v>
+        <x:v>1. Qualifier Android sur appareil, les comptes réels et les parcours sur les plateformes cibles.</x:v>
       </x:c>
       <x:c r="C29" s="2"/>
       <x:c r="D29" s="2"/>
@@ -1356,7 +1356,7 @@
         <x:v>Preuves dans le dépôt</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="48" customHeight="1">
+    <x:row r="8" ht="49" customHeight="1">
       <x:c r="A8" s="13" t="str">
         <x:v>FG-001</x:v>
       </x:c>
@@ -1364,7 +1364,7 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="C8" s="14" t="str">
-        <x:v>À valider</x:v>
+        <x:v>Terminé</x:v>
       </x:c>
       <x:c r="D8" s="11" t="str">
         <x:v>Livraison</x:v>
@@ -1376,7 +1376,7 @@
         <x:v>Importer la suite complète dans GitHub</x:v>
       </x:c>
       <x:c r="G8" s="12" t="str">
-        <x:v>Archive V0.35 récupérée et copiée dans le dépôt local. Le dépôt distant initial ne contenait que le README.</x:v>
+        <x:v>Suite publiée sur main dans le dépôt demandé. Le premier commit applicatif vérifié contient 589 fichiers, dont les sources et le classeur.</x:v>
       </x:c>
       <x:c r="H8" s="12" t="str">
         <x:v>Publier les sources Android, Web, PC, tests, outils et documentation en conservant les notices. Contrôler l’arbre distant après publication.</x:v>
@@ -1388,14 +1388,14 @@
         <x:v>Aucune</x:v>
       </x:c>
       <x:c r="K8" s="12" t="str">
-        <x:v>Non vérifié dans cette passe</x:v>
+        <x:v>Commit f954889bceaa81636c5c24a37f78a5ea1951554c retrouvé dans un nouveau clone public propre. Arbre et Excel vérifiés.</x:v>
       </x:c>
       <x:c r="L8" s="15" t="str"/>
       <x:c r="M8" s="12" t="str">
-        <x:v>README.md; RELEASE.json; MANIFEST.sha256</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="62" customHeight="1">
+        <x:v>README.md; docs/INTEGRATION_GITHUB.md; RELEASE.json; MANIFEST.sha256</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="88" customHeight="1">
       <x:c r="A9" s="13" t="str">
         <x:v>FG-002</x:v>
       </x:c>
@@ -1415,7 +1415,7 @@
         <x:v>Exécuter les contrôles à chaque modification</x:v>
       </x:c>
       <x:c r="G9" s="12" t="str">
-        <x:v>Workflow push/PR ajouté dans cette passe. Dépendances verrouillées et commandes de vérification définies. L’exécution GitHub de la version finale reste à observer.</x:v>
+        <x:v>Workflow push/PR publié et exécuté. Groupes Web/PC et Android distants réussis. Le test navigateur corrigé réussit localement sur la version Chromium de CI et sur Chrome 156 ; sa nouvelle exécution distante reste à observer.</x:v>
       </x:c>
       <x:c r="H9" s="12" t="str">
         <x:v>Déclencher la CI sur push et PR. Installer les dépendances verrouillées et exécuter les suites appropriées, avec journaux et artefacts.</x:v>
@@ -1427,11 +1427,13 @@
         <x:v>FG-001</x:v>
       </x:c>
       <x:c r="K9" s="12" t="str">
-        <x:v>Non vérifié dans cette passe</x:v>
-      </x:c>
-      <x:c r="L9" s="15" t="str"/>
+        <x:v>Web/PC : GitHub Actions 40402158558 réussi. Android : job 121851777726 du run 40402512586 réussi, APK et rapports publiés. ChromeHeadlessShell 151 et Chrome 156 : 22/22 contrôles chacun après correction du test ; correction navigateur à republier.</x:v>
+      </x:c>
+      <x:c r="L9" s="15" t="str">
+        <x:v>L’injection contrôlée de régression reste à exercer pour fermer le critère. La divergence navigator.onLine est un diagnostic navigateur ; la preuve hors ligne utilise désormais le rejet réel d’une requête sans cache.</x:v>
+      </x:c>
       <x:c r="M9" s="12" t="str">
-        <x:v>.github/workflows/build.yml; package.json</x:v>
+        <x:v>.github/workflows/build.yml; package.json; docs/QA_REPORT.md; docs/qa/current.json</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="101" customHeight="1">
@@ -1454,7 +1456,7 @@
         <x:v>Compiler réellement Android avec SDK et Compose</x:v>
       </x:c>
       <x:c r="G10" s="12" t="str">
-        <x:v>SDK36 installé. compileDebugKotlin réussit après correction de trois fichiers Compose invalides dans la base. Assemblage APK et lint en cours.</x:v>
+        <x:v>Compilation SDK/Compose, assemblage de l’APK et lint réussis. Trois fichiers Compose invalides et 13 erreurs lint corrigés. Les tests Android JUnit ne sont pas encore présents.</x:v>
       </x:c>
       <x:c r="H10" s="12" t="str">
         <x:v>Exécuter assembleDebug, tests unitaires et lint avec JDK17 et SDK requis. Corriger les erreurs et conserver les rapports.</x:v>
@@ -1466,14 +1468,16 @@
         <x:v>FG-002</x:v>
       </x:c>
       <x:c r="K10" s="12" t="str">
-        <x:v>compileDebugKotlin réel réussi (3 min 16 s). Corrections de blocs/lambda/import Job et argument par défaut. assembleDebug, testDebugUnitTest et lintDebug encore en cours. Aucun essai appareil.</x:v>
-      </x:c>
-      <x:c r="L10" s="15" t="str"/>
+        <x:v>Local : assembleDebug + testDebugUnitTest + lintDebug, exit 0 en 5 min 24 s. CI Android : même groupe réussi en 5 min 55 s. Lint : 0 erreur, 31 avertissements, 1 remarque. JUnit Android : NO-SOURCE, aucun test exécuté. APK debug v2 vérifiée.</x:v>
+      </x:c>
+      <x:c r="L10" s="15" t="str">
+        <x:v>Complément pour clore le critère de tests : ajouter/exécuter de vrais tests unitaires Android. Les 31 avertissements lint ne sont pas 31 bugs fonctionnels : 21 UseKtx, 6 dépendances, 1 ApplySharedPref, 1 ObsoleteSdkInt, 1 Overdraw et 1 HardcodedText. Préserver le commit synchrone requis par la sécurité.</x:v>
+      </x:c>
       <x:c r="M10" s="12" t="str">
-        <x:v>app/build.gradle.kts; build.gradle.kts; app/src/main/java/com/franchiseguide/app/ui/FranchisePanels.kt; app/src/main/java/com/franchiseguide/app/ui/InsightsPanels.kt; app/src/main/java/com/franchiseguide/app/ui/WatchAvailabilityScreen.kt; docs/ANDROID_BUILD.md</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="62" customHeight="1">
+        <x:v>app/build.gradle.kts; build.gradle.kts; app/src/main/java/com/franchiseguide/app/ui/FranchisePanels.kt; app/src/main/java/com/franchiseguide/app/ui/InsightsPanels.kt; app/src/main/java/com/franchiseguide/app/ui/WatchAvailabilityScreen.kt; docs/ANDROID_BUILD.md; docs/qa/current.json</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="49" customHeight="1">
       <x:c r="A11" s="13" t="str">
         <x:v>FG-004</x:v>
       </x:c>
@@ -1481,7 +1485,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C11" s="14" t="str">
-        <x:v>Partiel</x:v>
+        <x:v>Terminé</x:v>
       </x:c>
       <x:c r="D11" s="11" t="str">
         <x:v>Livraison</x:v>
@@ -1493,7 +1497,7 @@
         <x:v>Harmoniser versions et manifestes de distribution</x:v>
       </x:c>
       <x:c r="G11" s="12" t="str">
-        <x:v>Versions source, npm, Android, cache et manifest harmonisées en 0.36.0. Miroirs Web synchronisés et JAR PC reconstruit. Vérification du manifeste final après export Excel à terminer.</x:v>
+        <x:v>Versions harmonisées en 0.36.0, miroirs Web synchronisés et JAR PC reconstruit. Le manifeste du premier clone publié a été vérifié.</x:v>
       </x:c>
       <x:c r="H11" s="12" t="str">
         <x:v>Synchroniser les métadonnées, reconstruire le JAR, générer les empreintes et comparer les ressources des distributions.</x:v>
@@ -1505,14 +1509,16 @@
         <x:v>FG-001</x:v>
       </x:c>
       <x:c r="K11" s="12" t="str">
-        <x:v>JAR 0.36.0 et --probe réussis. 109 contrôles HTTP + 9 de démarrage. Copies Web vérifiées par l’intégration. Empreintes finales à régénérer après cet export.</x:v>
-      </x:c>
-      <x:c r="L11" s="15" t="str"/>
+        <x:v>588 fichiers SHA-256 vérifiés dans le clone public. JAR 0.36.0 et --probe réussis ; 109 contrôles HTTP et 9 de démarrage.</x:v>
+      </x:c>
+      <x:c r="L11" s="15" t="str">
+        <x:v>Régénérer le manifeste après chaque nouvelle modification ou export du classeur.</x:v>
+      </x:c>
       <x:c r="M11" s="12" t="str">
         <x:v>tools/build_pc.sh; web/sw.js; web/manifest.webmanifest; RELEASE.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="49" customHeight="1">
+    <x:row r="12" ht="62" customHeight="1">
       <x:c r="A12" s="13" t="str">
         <x:v>FG-005</x:v>
       </x:c>
@@ -1520,7 +1526,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C12" s="14" t="str">
-        <x:v>Partiel</x:v>
+        <x:v>Terminé</x:v>
       </x:c>
       <x:c r="D12" s="11" t="str">
         <x:v>Livraison</x:v>
@@ -1532,7 +1538,7 @@
         <x:v>Consolider la documentation courante</x:v>
       </x:c>
       <x:c r="G12" s="12" t="str">
-        <x:v>Plusieurs guides décrivent encore V0.14/V0.22 et schéma8 alors que le portable courant est V11. Les barrières de publication datent de V0.29.</x:v>
+        <x:v>Entrées README/START_HERE, matrice, barrières de publication et guide Android actualisés. Quatre guides liés clarifient 0.36.0, portable 11 et preuves historiques.</x:v>
       </x:c>
       <x:c r="H12" s="12" t="str">
         <x:v>Séparer les références historiques des instructions courantes. Mettre à jour matrice de fonctions, conditions de démarrage et barrières selon preuves de cette passe.</x:v>
@@ -1544,14 +1550,14 @@
         <x:v>FG-004</x:v>
       </x:c>
       <x:c r="K12" s="12" t="str">
-        <x:v>Non vérifié dans cette passe</x:v>
+        <x:v>Lecture des guides liés. Contradictions « export courant schéma 8 » et « aucun build SDK » supprimées. Le rapport QA courant reste la référence des résultats.</x:v>
       </x:c>
       <x:c r="L12" s="15" t="str"/>
       <x:c r="M12" s="12" t="str">
-        <x:v>docs/RELEASE_GATES.json; docs/ANDROID_BUILD.md; docs/GAMING_ACHIEVEMENTS.md; docs/FEATURE_MATRIX.md</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="49" customHeight="1">
+        <x:v>README.md; START_HERE.md; docs/FEATURE_MATRIX.md; docs/GAMING_ACHIEVEMENTS.md; docs/STEAM_SIGN_IN.md; docs/RETROACHIEVEMENTS.md; docs/PRIVACY_TECHNICAL.md</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="75" customHeight="1">
       <x:c r="A13" s="13" t="str">
         <x:v>FG-006</x:v>
       </x:c>
@@ -1559,7 +1565,7 @@
         <x:v>P1</x:v>
       </x:c>
       <x:c r="C13" s="14" t="str">
-        <x:v>À valider</x:v>
+        <x:v>Terminé</x:v>
       </x:c>
       <x:c r="D13" s="11" t="str">
         <x:v>Livraison</x:v>
@@ -1571,10 +1577,10 @@
         <x:v>Reproduire la suite depuis un clone vierge</x:v>
       </x:c>
       <x:c r="G13" s="12" t="str">
-        <x:v>Scripts de bootstrap, compilation PC et tests présents. L’archive comprend des sorties de tests historiques.</x:v>
+        <x:v>Nouveau clone public sans modification locale exercé après publication. Les dépendances ont été installées depuis le lockfile en utilisant le cache npm du poste.</x:v>
       </x:c>
       <x:c r="H13" s="12" t="str">
-        <x:v>Documenter et exercer un parcours propre sur machine sans caches. Contrôler exclusions Git, permissions des scripts et dépendances téléchargées.</x:v>
+        <x:v>Cloner dans un répertoire vierge, installer les dépendances verrouillées avec les prérequis documentés, exercer la structure, le build PC et le démarrage Web. Documenter les caches réutilisés.</x:v>
       </x:c>
       <x:c r="I13" s="12" t="str">
         <x:v>Clone vierge puis commandes documentées suffisants pour lancer Web et construire PC. Échecs de prérequis expliqués.</x:v>
@@ -1583,9 +1589,11 @@
         <x:v>FG-002</x:v>
       </x:c>
       <x:c r="K13" s="12" t="str">
-        <x:v>Non vérifié dans cette passe</x:v>
-      </x:c>
-      <x:c r="L13" s="15" t="str"/>
+        <x:v>HEAD exact et arbre propre. npm ci --offline : 42 paquets. Structure : 216 contrôles. Build PC et --probe réussis. npm start répond HTTP 200 sur port 47642.</x:v>
+      </x:c>
+      <x:c r="L13" s="15" t="str">
+        <x:v>Cette recette réutilise le cache npm de l’environnement. La CI distante vérifie séparément le parcours d’installation sur son runner.</x:v>
+      </x:c>
       <x:c r="M13" s="12" t="str">
         <x:v>tools/bootstrap-gradle.sh; tools/build_pc.sh; tools/run_checks.sh; package-lock.json</x:v>
       </x:c>
@@ -2175,7 +2183,7 @@
         <x:v>web/manifest.webmanifest; web/sw.js; docs/WEB.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="29" ht="62" customHeight="1">
+    <x:row r="29" ht="75" customHeight="1">
       <x:c r="A29" s="13" t="str">
         <x:v>FG-022</x:v>
       </x:c>
@@ -2195,7 +2203,7 @@
         <x:v>Vérifier le démarrage hors ligne</x:v>
       </x:c>
       <x:c r="G29" s="12" t="str">
-        <x:v>Moteur et caches présents. Rechargement hors ligne vérifié sur origine HTTP réelle dans Chrome 156, avec stockage réel. Autres navigateurs et installation OS restent à tester.</x:v>
+        <x:v>Rechargement hors ligne et stockage réel vérifiés sur origine HTTP dans Chrome 156 et ChromeHeadlessShell 151 (version CI). Autres navigateurs et installation OS restent à tester.</x:v>
       </x:c>
       <x:c r="H29" s="12" t="str">
         <x:v>Tester démarrage à froid après installation, navigation en mode avion et données sans image. Rendre les opérations indisponibles explicites.</x:v>
@@ -2207,11 +2215,11 @@
         <x:v>FG-021</x:v>
       </x:c>
       <x:c r="K29" s="12" t="str">
-        <x:v>tests/browser-origin.cjs : rechargement hors ligne et absence d’API privées dans les caches vérifiés dans le groupe de 22 contrôles réussis. Pas de PWA installée OS.</x:v>
+        <x:v>22/22 contrôles sur chacune des deux versions Chrome. URL à nonce : HTTP 404 en ligne, fetch rejeté hors ligne sans cache ; rechargement servi par le service worker, 4 titres et thème conservés en mémoire et localStorage. Pas de PWA installée OS.</x:v>
       </x:c>
       <x:c r="L29" s="15" t="str"/>
       <x:c r="M29" s="12" t="str">
-        <x:v>web/sw.js; web/maintenance.js; tests/sw.test.cjs; tests/browser-origin.cjs</x:v>
+        <x:v>web/sw.js; web/maintenance.js; tests/sw.test.cjs; tests/browser-origin.cjs; docs/qa/current.json</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="48" customHeight="1">
@@ -2273,7 +2281,7 @@
         <x:v>Éprouver stockage persistant, quotas et éviction</x:v>
       </x:c>
       <x:c r="G31" s="12" t="str">
-        <x:v>Copies IndexedDB et contrôles de persistance présents. Les tests récupérés n’établissent pas le comportement d’une origine persistante réelle.</x:v>
+        <x:v>Copies IndexedDB et contrôles de persistance présents. localStorage et IndexedDB exercés sur une origine réelle Chrome ; quotas, permission de persistance et éviction restent non qualifiés.</x:v>
       </x:c>
       <x:c r="H31" s="12" t="str">
         <x:v>Tester navigateurs ordinaires/privés, quota plein, permission de persistance et suppression de données du site.</x:v>
@@ -2285,11 +2293,11 @@
         <x:v>FG-021</x:v>
       </x:c>
       <x:c r="K31" s="12" t="str">
-        <x:v>Stockages localStorage et IndexedDB réels exercés dans Chrome 156. Quota plein, persistance accordée/refusée, mode privé et éviction restent à vérifier.</x:v>
+        <x:v>Stockages localStorage et IndexedDB réels exercés dans Chrome 156 et ChromeHeadlessShell 151. Quota plein, persistance accordée/refusée, mode privé et éviction restent à vérifier.</x:v>
       </x:c>
       <x:c r="L31" s="15" t="str"/>
       <x:c r="M31" s="12" t="str">
-        <x:v>web/durable.js; web/persistence.js; web/maintenance.js; tests/browser-origin.cjs</x:v>
+        <x:v>web/durable.js; web/persistence.js; web/maintenance.js; tests/browser-origin.cjs; docs/qa/current.json</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="62" customHeight="1">
@@ -2312,7 +2320,7 @@
         <x:v>Vérifier les conflits de deux fenêtres réelles</x:v>
       </x:c>
       <x:c r="G32" s="12" t="str">
-        <x:v>Verrou entre deux onglets et transfert de contrôle exercés sur origine réelle Chrome 156. La matrice de conflits complexes et autres moteurs reste ouverte.</x:v>
+        <x:v>Verrou entre deux onglets et transfert de contrôle exercés sur origine réelle dans Chrome 156 et ChromeHeadlessShell 151. Les conflits complexes et autres moteurs restent ouverts.</x:v>
       </x:c>
       <x:c r="H32" s="12" t="str">
         <x:v>Modifier le même média, importer et synchroniser dans deux fenêtres. Implémenter un verrou ou une résolution conservatrice si nécessaire.</x:v>
@@ -2324,11 +2332,11 @@
         <x:v>FG-021</x:v>
       </x:c>
       <x:c r="K32" s="12" t="str">
-        <x:v>tests/browser-origin.cjs : deux onglets, lecture seule et transfert du verrou vérifiés. Scénarios avancés de concurrence et autres navigateurs à compléter.</x:v>
+        <x:v>Dans le groupe de 22 contrôles réussi sur chaque version Chrome : deux onglets, lecture seule et transfert du verrou. Scénarios avancés de concurrence et autres moteurs à compléter.</x:v>
       </x:c>
       <x:c r="L32" s="15" t="str"/>
       <x:c r="M32" s="12" t="str">
-        <x:v>web/persistence.js; web/reliability-core.js; web/import-ui.js; tests/browser-origin.cjs</x:v>
+        <x:v>web/persistence.js; web/reliability-core.js; web/import-ui.js; tests/browser-origin.cjs; docs/qa/current.json</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="48" customHeight="1">
@@ -2448,7 +2456,7 @@
         <x:v>web/app.css; app/src/main/java/com/franchiseguide/app/ui/theme/Theme.kt</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="49" customHeight="1">
+    <x:row r="36" ht="62" customHeight="1">
       <x:c r="A36" s="13" t="str">
         <x:v>FG-029</x:v>
       </x:c>
@@ -2468,7 +2476,7 @@
         <x:v>Parcourir les écrans sur téléphone et grand écran</x:v>
       </x:c>
       <x:c r="G36" s="12" t="str">
-        <x:v>Des captures historiques couvrent plusieurs largeurs, sans preuve complète de cette version sur appareils.</x:v>
+        <x:v>Écran Web contrôlé à 390 px dans Chrome réel, sans débordement. La matrice de tailles, les claviers virtuels et les appareils Android restent à qualifier.</x:v>
       </x:c>
       <x:c r="H36" s="12" t="str">
         <x:v>Exercer petites largeurs, paysage, écrans tactiles et grandes bibliothèques. Corriger débordements, menus et champs masqués.</x:v>
@@ -2480,11 +2488,11 @@
         <x:v>FG-009</x:v>
       </x:c>
       <x:c r="K36" s="12" t="str">
-        <x:v>Chrome 156 à 390 px sans débordement dans tests/browser-origin.cjs. Autres largeurs, paysage, clavier virtuel et Android appareil à compléter.</x:v>
+        <x:v>Chrome 156 et ChromeHeadlessShell 151 à 390 px sans débordement dans tests/browser-origin.cjs. Autres largeurs, paysage, clavier virtuel et Android appareil à compléter.</x:v>
       </x:c>
       <x:c r="L36" s="15" t="str"/>
       <x:c r="M36" s="12" t="str">
-        <x:v>web/app.css; web/views.js; app/src/main/java/com/franchiseguide/app/ui/</x:v>
+        <x:v>web/app.css; web/views.js; app/src/main/java/com/franchiseguide/app/ui/; docs/qa/current.json</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="48" customHeight="1">
@@ -4983,7 +4991,7 @@
         <x:v>app/build.gradle.kts; docs/ANDROID_BUILD.md; docs/RELEASE_GATES.json</x:v>
       </x:c>
     </x:row>
-    <x:row r="101" ht="49" customHeight="1">
+    <x:row r="101" ht="88" customHeight="1">
       <x:c r="A101" s="13" t="str">
         <x:v>FG-094</x:v>
       </x:c>
@@ -5015,11 +5023,11 @@
         <x:v>FG-002, FG-003, FG-021, FG-082</x:v>
       </x:c>
       <x:c r="K101" s="12" t="str">
-        <x:v>npm test : 1 580/1 580, 0 échec, 0 ignoré. Structure : 216 contrôles. Passerelles Java : 353 assertions. Origine Chrome 156 : 22 contrôles. Comptes réels et matrice complète non exécutés.</x:v>
+        <x:v>Node : 1 580/1 580, 0 échec/ignoré. Structure : 216. Passerelles Java : 353 assertions. Navigateurs : 22/22 sur Chrome 156 et ChromeHeadlessShell 151. Kotlin check-in : 33 assertions + parité. SDK/APK/lint réussis localement et en CI ; JUnit Android NO-SOURCE. Relance navigateur distante à observer.</x:v>
       </x:c>
       <x:c r="L101" s="15" t="str"/>
       <x:c r="M101" s="12" t="str">
-        <x:v>docs/QA_REPORT.md; tests/browser-origin.cjs; tools/validate_project.py; docs/RELEASE_GATES.json</x:v>
+        <x:v>docs/QA_REPORT.md; tests/browser-origin.cjs; tools/validate_project.py; docs/RELEASE_GATES.json; docs/qa/current.json</x:v>
       </x:c>
     </x:row>
     <x:row r="102" ht="49" customHeight="1">
@@ -5217,7 +5225,7 @@
         <x:v>server/steam-bridge.cjs; desktop/src/com/franchiseguide/desktop/SteamBridge.java</x:v>
       </x:c>
     </x:row>
-    <x:row r="107" ht="49" customHeight="1">
+    <x:row r="107" ht="62" customHeight="1">
       <x:c r="A107" s="13" t="str">
         <x:v>FG-100</x:v>
       </x:c>
@@ -5249,14 +5257,14 @@
         <x:v>Aucune</x:v>
       </x:c>
       <x:c r="K107" s="12" t="str">
-        <x:v>Tests de reprise V0.36 : 33/33. Tests check-in V0.35 : 23/23. Fournisseurs et stockage simulés. Portage Android en sources, validation native séparée.</x:v>
+        <x:v>Web : reprise V0.36 33/33, check-in V0.35 23/23. Kotlin/JVM : 33 assertions et parité JS/Kotlin réussies. Fournisseurs simulés. Compte réel et appareil non testés.</x:v>
       </x:c>
       <x:c r="L107" s="15" t="str"/>
       <x:c r="M107" s="12" t="str">
         <x:v>web/trakt-checkin-core.js; web/trakt-checkin-ui.js; tests/checkin-recovery-v036.test.cjs; tests/checkin-v035.test.cjs</x:v>
       </x:c>
     </x:row>
-    <x:row r="108" ht="49" customHeight="1">
+    <x:row r="108" ht="62" customHeight="1">
       <x:c r="A108" s="13" t="str">
         <x:v>FG-101</x:v>
       </x:c>
@@ -5288,7 +5296,7 @@
         <x:v>Aucune</x:v>
       </x:c>
       <x:c r="K108" s="12" t="str">
-        <x:v>Tests de reprise V0.36 : 33/33. Tests check-in V0.35 : 23/23. Fournisseurs et stockage simulés. Portage Android en sources, validation native séparée.</x:v>
+        <x:v>Web : reprise V0.36 33/33, check-in V0.35 23/23. Kotlin/JVM : 33 assertions et parité JS/Kotlin réussies. Fournisseurs simulés. Compte réel et appareil non testés.</x:v>
       </x:c>
       <x:c r="L108" s="15" t="str"/>
       <x:c r="M108" s="12" t="str">
@@ -5327,14 +5335,14 @@
         <x:v>Aucune</x:v>
       </x:c>
       <x:c r="K109" s="12" t="str">
-        <x:v>Web : reprise 33/33 et check-in 23/23. Correction de lecture JSON Android portée en source, compilation/tests natifs en cours. Aucun essai appareil revendiqué.</x:v>
+        <x:v>Web : reprise 33/33 et check-in 23/23. Kotlin/JVM règles : 33 assertions et parité réussies. Codec nullable Android corrigé et compilé, sans test de lecture JSON natif ni essai appareil.</x:v>
       </x:c>
       <x:c r="L109" s="15" t="str"/>
       <x:c r="M109" s="12" t="str">
         <x:v>web/trakt-checkin-ui.js; tests/checkin-recovery-v036.test.cjs; app/src/main/java/com/franchiseguide/app/data/AppRepository.kt</x:v>
       </x:c>
     </x:row>
-    <x:row r="110" ht="49" customHeight="1">
+    <x:row r="110" ht="62" customHeight="1">
       <x:c r="A110" s="13" t="str">
         <x:v>FG-103</x:v>
       </x:c>
@@ -5366,7 +5374,7 @@
         <x:v>Aucune</x:v>
       </x:c>
       <x:c r="K110" s="12" t="str">
-        <x:v>Tests de reprise V0.36 : 33/33. Tests check-in V0.35 : 23/23. Fournisseurs et stockage simulés. Portage Android en sources, validation native séparée.</x:v>
+        <x:v>Web : reprise V0.36 33/33, check-in V0.35 23/23. Kotlin/JVM : 33 assertions et parité JS/Kotlin réussies. Fournisseurs simulés. Compte réel et appareil non testés.</x:v>
       </x:c>
       <x:c r="L110" s="15" t="str"/>
       <x:c r="M110" s="12" t="str">
@@ -5409,7 +5417,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4be754086724595"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41b6e8a78669473b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>